<commit_message>
Add plot shapes with fill opacity, Caps Lock-safe undo, and version archive.
Rectangle/square/circle tools use the colour picker plus an opacity slider; undo/redo keeps working after drawing; changelog and MongoDB-backed archive tooling start at v1.3.0.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ShyamGui/CHANGELOG.xlsx
+++ b/ShyamGui/CHANGELOG.xlsx
@@ -1,20 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.0 Changes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.1.0 Changes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.0.0 Baseline" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="v1.3.0 Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="v1.1.0 Changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="v1.0.0 Baseline" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="Timeline" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'v1.3.0 Changes'!$A$4:$E$17</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'v1.3.0 Changes'!$A$4:$E$24</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'v1.1.0 Changes'!$A$4:$E$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -605,17 +605,17 @@
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Windows product + drawing tools</t>
+          <t>Q21S BEM heatmap + Windows/mac product</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>ATOMIK-only branding, v1.3.0 exe, plot pencil/line/ruler/eraser, BEM/directivity math, Ctrl+Z/Y undo-redo, Statistics button, header version fix</t>
+          <t>BEM polar×1/r full-grid SPL, cardioid preset, Q21S 750×784×917 mm, plot tools, undo/redo, ATOMIK branding, heatmap docs/zip, version archive</t>
         </is>
       </c>
     </row>
@@ -690,7 +690,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E19"/>
+  <dimension ref="A1:E26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -714,7 +714,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Development window 2026-08-12 -&gt; 2026-08-19</t>
+          <t>Development window 2026-08-12 -&gt; 2026-08-21</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -759,7 +759,7 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>Plot tools</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="B5" s="9" t="inlineStr">
@@ -769,24 +769,24 @@
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Heatmap drawing tools</t>
+          <t>Q21S BEM polar × 1/r SPL</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Select, Pan, Pencil, Eraser, Ruler, Line + colour swatch; annotations in world metres</t>
+          <t>Far-field (~2 m) D(θ) coherent complex sum; r_spread floored at cabinet half-depth; absolute dB SPL from on-axis BEM; no ±5 m field stamp</t>
         </is>
       </c>
       <c r="E5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>Plot tools</t>
+          <t>Array presets</t>
         </is>
       </c>
       <c r="B6" s="10" t="inlineStr">
@@ -796,24 +796,24 @@
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>BEM / directivity field math</t>
+          <t>MATLAB-style cardioid</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Tightened BEM and measured-directivity field formation (commit 633fc36)</t>
+          <t>Rear 180°, polarity −1, −6 dB, 3.5 ms, ~0.01 m spacing; coherent engine sum</t>
         </is>
       </c>
       <c r="E6" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Editing</t>
+          <t>Docs / pack</t>
         </is>
       </c>
       <c r="B7" s="9" t="inlineStr">
@@ -823,24 +823,24 @@
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Undo / redo</t>
+          <t>Single-sub heatmap pack</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+Z, Ctrl+Y, Ctrl+Shift+Z; letter is lowercased so Caps Lock still works; drawings, cabinets, layouts, control-panel edits</t>
+          <t>docs/SINGLE_SUB_HEATMAP.md, native-Hz figures, generator script, dist_packages zip</t>
         </is>
       </c>
       <c r="E7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>Packaging</t>
+          <t>Archive</t>
         </is>
       </c>
       <c r="B8" s="10" t="inlineStr">
@@ -850,24 +850,24 @@
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Windows Release exe</t>
+          <t>Version archive (HTML + MongoDB)</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Builds\Release\Atomik Simulation Engine.exe; installer/README at v1.3.0</t>
+          <t>version-archive/: list releases from v1.3.0; download source zip / macOS DMG / Windows EXE (standalone, not in-app)</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>DSP / UI (PS batch)</t>
+          <t>Plot tools</t>
         </is>
       </c>
       <c r="B9" s="9" t="inlineStr">
@@ -877,39 +877,39 @@
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>IEC 1/3-octave frequencies</t>
+          <t>Heatmap drawing tools</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>20, 25, 31, 40, 50, 63, 80, 100, 125, 160, 200, 250, 315, 400, 500 Hz</t>
+          <t>Select, Pan, Pencil, Eraser, Ruler, Line + colour swatch; annotations in world metres</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
-          <t>Branding</t>
-        </is>
-      </c>
-      <c r="B10" s="11" t="inlineStr">
-        <is>
-          <t>Changed</t>
+          <t>Plot tools</t>
+        </is>
+      </c>
+      <c r="B10" s="10" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>Product name</t>
+          <t>BEM / directivity field math</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Atomik Acoustic Simulation Engine -&gt; Atomik Simulation Engine; UI/PDF/CSV/installer/file version = v1.3.0</t>
+          <t>Tightened BEM and measured-directivity field formation (commit 633fc36)</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -921,22 +921,22 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Branding</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>Changed</t>
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="B11" s="9" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>ATOMIK-only wordmark</t>
+          <t>Undo / redo</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>AUDIO line removed; Atomik_Logo_Dark.png / Atomik_Logo_Light.png</t>
+          <t>Ctrl+Z, Ctrl+Y, Ctrl+Shift+Z; letter is lowercased so Caps Lock still works; drawings, cabinets, layouts, control-panel edits</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
@@ -948,22 +948,22 @@
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Header</t>
-        </is>
-      </c>
-      <c r="B12" s="11" t="inlineStr">
-        <is>
-          <t>Changed</t>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B12" s="10" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Statistics button</t>
+          <t>Windows Release exe</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Stats pill renamed Statistics; width sized to the full label</t>
+          <t>Builds\Release\Atomik Simulation Engine.exe; installer/README at v1.3.0</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -975,22 +975,22 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>Measurement</t>
-        </is>
-      </c>
-      <c r="B13" s="12" t="inlineStr">
-        <is>
-          <t>Changed</t>
+          <t>DSP / UI (PS batch)</t>
+        </is>
+      </c>
+      <c r="B13" s="9" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>Ground Plane only</t>
+          <t>IEC 1/3-octave frequencies</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>Measurement UI is Ground Plane (no Room set in live UI)</t>
+          <t>20, 25, 31, 40, 50, 63, 80, 100, 125, 160, 200, 250, 315, 400, 500 Hz</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
@@ -1002,7 +1002,7 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>DSP</t>
+          <t>Cabinet</t>
         </is>
       </c>
       <c r="B14" s="11" t="inlineStr">
@@ -1012,24 +1012,24 @@
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Legend / dB floor -6 dB steps</t>
+          <t>Q21S footprint 750×784×917 mm</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Colourbar ticks and floor slider on -6 dB; dBfloor is display range only</t>
+          <t>Plan drawing + hit-test use true W×D; 1/r singularity floor = depth/2</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="B15" s="12" t="inlineStr">
@@ -1039,39 +1039,39 @@
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>XN18-n labels + Set to Default</t>
+          <t>Heatmap uses 2 m BEM arc</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Cabinet labels use hyphen; Reset renamed Set to Default</t>
+          <t>Array/SPL prediction keeps far-field arc; Measured Polar can still show nearer distances</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Header</t>
-        </is>
-      </c>
-      <c r="B16" s="13" t="inlineStr">
-        <is>
-          <t>Fixed</t>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="B16" s="11" t="inlineStr">
+        <is>
+          <t>Changed</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Version no longer clips</t>
+          <t>Product name</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Was showing v1... instead of v1.3.0; layout uses real logo width</t>
+          <t>Atomik Acoustic Simulation Engine -&gt; Atomik Simulation Engine; UI/PDF/CSV/installer/file version = v1.3.0</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
@@ -1083,46 +1083,235 @@
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="B17" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C17" s="6" t="inlineStr">
+        <is>
+          <t>ATOMIK-only wordmark</t>
+        </is>
+      </c>
+      <c r="D17" s="6" t="inlineStr">
+        <is>
+          <t>AUDIO line removed; Atomik_Logo_Dark.png / Atomik_Logo_Light.png</t>
+        </is>
+      </c>
+      <c r="E17" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="7" t="inlineStr">
+        <is>
+          <t>Header</t>
+        </is>
+      </c>
+      <c r="B18" s="11" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C18" s="8" t="inlineStr">
+        <is>
+          <t>Statistics button</t>
+        </is>
+      </c>
+      <c r="D18" s="8" t="inlineStr">
+        <is>
+          <t>Stats pill renamed Statistics; width sized to the full label</t>
+        </is>
+      </c>
+      <c r="E18" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="19">
+      <c r="A19" s="5" t="inlineStr">
+        <is>
+          <t>Measurement</t>
+        </is>
+      </c>
+      <c r="B19" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C19" s="6" t="inlineStr">
+        <is>
+          <t>Ground Plane only</t>
+        </is>
+      </c>
+      <c r="D19" s="6" t="inlineStr">
+        <is>
+          <t>Measurement UI is Ground Plane (no Room set in live UI)</t>
+        </is>
+      </c>
+      <c r="E19" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="7" t="inlineStr">
+        <is>
+          <t>DSP</t>
+        </is>
+      </c>
+      <c r="B20" s="11" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C20" s="8" t="inlineStr">
+        <is>
+          <t>Legend / dB floor -6 dB steps</t>
+        </is>
+      </c>
+      <c r="D20" s="8" t="inlineStr">
+        <is>
+          <t>Colourbar ticks and floor slider on -6 dB; dBfloor is display range only</t>
+        </is>
+      </c>
+      <c r="E20" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="5" t="inlineStr">
+        <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C21" s="6" t="inlineStr">
+        <is>
+          <t>XN18-n labels + Set to Default</t>
+        </is>
+      </c>
+      <c r="D21" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet labels use hyphen; Reset renamed Set to Default</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="7" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="C17" s="6" t="inlineStr">
+      <c r="C22" s="8" t="inlineStr">
+        <is>
+          <t>No ±5 m BEM stamp on live map</t>
+        </is>
+      </c>
+      <c r="D22" s="8" t="inlineStr">
+        <is>
+          <t>Full 100×100 m map follows polar × inverse-square instead of a near-field island</t>
+        </is>
+      </c>
+      <c r="E22" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="5" t="inlineStr">
+        <is>
+          <t>Header</t>
+        </is>
+      </c>
+      <c r="B23" s="14" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C23" s="6" t="inlineStr">
+        <is>
+          <t>Version no longer clips</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>Was showing v1... instead of v1.3.0; layout uses real logo width</t>
+        </is>
+      </c>
+      <c r="E23" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B24" s="13" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
         <is>
           <t>Small-screen logo</t>
         </is>
       </c>
-      <c r="D17" s="6" t="inlineStr">
+      <c r="D24" s="8" t="inlineStr">
         <is>
           <t>Header/dashboard wordmark -20%; Scale minFactor 0.78</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr">
+      <c r="E24" s="8" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="A18" s="2" t="n"/>
-      <c r="B18" s="2" t="n"/>
-      <c r="C18" s="2" t="n"/>
-      <c r="D18" s="2" t="n"/>
-      <c r="E18" s="2" t="n"/>
-    </row>
-    <row r="19">
-      <c r="A19" s="2" t="n"/>
-      <c r="B19" s="2" t="n"/>
-      <c r="C19" s="2" t="n"/>
-      <c r="D19" s="2" t="n"/>
-      <c r="E19" s="2" t="n"/>
+    <row r="25">
+      <c r="A25" s="2" t="n"/>
+      <c r="B25" s="2" t="n"/>
+      <c r="C25" s="2" t="n"/>
+      <c r="D25" s="2" t="n"/>
+      <c r="E25" s="2" t="n"/>
+    </row>
+    <row r="26">
+      <c r="A26" s="2" t="n"/>
+      <c r="B26" s="2" t="n"/>
+      <c r="C26" s="2" t="n"/>
+      <c r="D26" s="2" t="n"/>
+      <c r="E26" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E17"/>
+  <autoFilter ref="A4:E24"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
@@ -2372,7 +2561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B16"/>
+  <dimension ref="A1:B17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2532,12 +2721,24 @@
       </c>
     </row>
     <row r="15">
-      <c r="A15" s="2" t="n"/>
-      <c r="B15" s="2" t="n"/>
+      <c r="A15" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>Q21S BEM polar×1/r, cardioid preset, cabinet size, heatmap docs/zip, version archive; CHANGELOG date → 2026-08-21</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" s="2" t="n"/>
       <c r="B16" s="2" t="n"/>
+    </row>
+    <row r="17">
+      <c r="A17" s="2" t="n"/>
+      <c r="B17" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Release v1.3.6: restore mic ring snap and shape-edge Snap tak.
Mic drag uses original Drag::Mic latch again; Snap tak fires when drawings meet edge-to-edge. Bump archive HTML/json and product version to 1.3.6.

Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ShyamGui/CHANGELOG.xlsx
+++ b/ShyamGui/CHANGELOG.xlsx
@@ -1,21 +1,25 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet name="v1.3.0 Changes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet name="v1.1.0 Changes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet name="v1.0.0 Baseline" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet name="Timeline" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.6 Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.5 Changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.0 Changes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.2.x Beta UI" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.1.0 Changes" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.0.0 Baseline" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'v1.3.0 Changes'!$A$4:$E$24</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'v1.1.0 Changes'!$A$4:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'v1.3.0 Changes'!$A$4:$E$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'v1.2.x Beta UI'!$A$4:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'v1.1.0 Changes'!$A$4:$E$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -63,6 +67,12 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
+      <color rgb="00FF6B6B"/>
+      <sz val="10"/>
+    </font>
+    <font>
+      <name val="Calibri"/>
+      <b val="1"/>
       <color rgb="0053D769"/>
       <sz val="10"/>
     </font>
@@ -70,12 +80,6 @@
       <name val="Calibri"/>
       <b val="1"/>
       <color rgb="0044D9E6"/>
-      <sz val="10"/>
-    </font>
-    <font>
-      <name val="Calibri"/>
-      <b val="1"/>
-      <color rgb="00FF6B6B"/>
       <sz val="10"/>
     </font>
   </fonts>
@@ -163,13 +167,13 @@
     <xf numFmtId="0" fontId="6" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
@@ -540,7 +544,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D9"/>
+  <dimension ref="A1:D12"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -600,80 +604,146 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>1.3.0</t>
+          <t>1.3.6</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Q21S BEM heatmap + Windows/mac product</t>
+          <t>Mic snap + shape-edge tak</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>BEM polar×1/r full-grid SPL, cardioid preset, Q21S 750×784×917 mm, plot tools, undo/redo, ATOMIK branding, heatmap docs/zip, version archive</t>
+          <t>Restored original mic Drag::Mic ring snap; tak when drawings meet edge-to-edge; start.md for build/run; v1.3.6 Windows Release</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>1.1.0</t>
+          <t>1.3.5</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Major feature + UX release</t>
+          <t>Mic tool + embedded Q21S Setup</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Theming, project dashboard/.atmk, heatmap + PDF export, grid/CAD-DXF, array presets, dual datasets, responsive window, branded installer</t>
+          <t>Virtual mics, FR floating window, Show Degrees, tak snap sound; Q21S CSVs baked into EXE; Windows Setup without Excel/Data folder</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
+          <t>1.3.0</t>
+        </is>
+      </c>
+      <c r="B7" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Q21S BEM heatmap + Windows/mac product</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>BEM polar×1/r full-grid SPL, cardioid, Q21S 750×784×917 mm, plot tools/shapes, undo/redo, ATOMIK branding, version archive, Windows portable ZIP (EXE+Data)</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>1.2.x</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="inlineStr">
+        <is>
+          <t>~2026-07</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Beta UI redesign (betav1.2.3)</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Graph colors.pdf chrome: brand tokens, heatmap colour stops, light/dark sidebar; packaged as betav1.2.3-style Release</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="B9" s="6" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Major feature + UX release</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Theming, project dashboard/.atmk, heatmap + PDF export, grid/CAD-DXF, array presets, dual datasets, responsive window, branded installer</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
           <t>1.0.0</t>
         </is>
       </c>
-      <c r="B7" s="6" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="C7" s="6" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Initial baseline</t>
         </is>
       </c>
-      <c r="D7" s="6" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Dual-subwoofer (XN18) prediction &amp; visualisation in a 30x30 m world; measured directivity added 2026-06-24</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="2" t="n"/>
-      <c r="B8" s="2" t="n"/>
-      <c r="C8" s="2" t="n"/>
-      <c r="D8" s="2" t="n"/>
-    </row>
-    <row r="9">
-      <c r="A9" s="2" t="n"/>
-      <c r="B9" s="2" t="n"/>
-      <c r="C9" s="2" t="n"/>
-      <c r="D9" s="2" t="n"/>
+    <row r="11">
+      <c r="A11" s="2" t="n"/>
+      <c r="B11" s="2" t="n"/>
+      <c r="C11" s="2" t="n"/>
+      <c r="D11" s="2" t="n"/>
+    </row>
+    <row r="12">
+      <c r="A12" s="2" t="n"/>
+      <c r="B12" s="2" t="n"/>
+      <c r="C12" s="2" t="n"/>
+      <c r="D12" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -690,7 +760,436 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E26"/>
+  <dimension ref="A1:E8"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>v1.3.6  -  Detailed Changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-31  |  Mic ring snap + shape-edge Snap tak</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Mic tool</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Original Drag::Mic ring snap</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Cursor-follow + 1/2/4/8 m latch + tak; no sticky lock from SelectionMove/object snap</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Plot Snap</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Tak when shapes meet</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Sound on rising edge of annotation edge contact; not speakers/mics/centres</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Docs</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>start.md</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Repo-root build/run instructions for Windows Debug/Release and MSBuild</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Version → v1.3.6</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>App, resource, installer defines, archive HTML/json</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-31</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E11"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>v1.3.5  -  Detailed Changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-08-26  |  Mic tool + embedded Q21S Windows Setup</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Mic tool</t>
+        </is>
+      </c>
+      <c r="B5" s="11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Virtual receivers on heatmap</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Add Mic / Place on ring; ring snap 1/2/4/8 m; live relative dB; Esc cancels arm</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Mic tool</t>
+        </is>
+      </c>
+      <c r="B6" s="13" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Show Degrees toggle</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Angle vs Q21S facing (0° = front, CCW) shown before dB on mic labels</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Mic tool</t>
+        </is>
+      </c>
+      <c r="B7" s="11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Floating Frequency Response window</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Opens when mics exist; does not shrink the plot; curves from sampleIntensityAt</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Mic tool</t>
+        </is>
+      </c>
+      <c r="B8" s="13" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Tak snap sound</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>In-memory WAV via winmm; no .wav asset on disk</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Embedded Q21S CSVs in EXE</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>EmbeddedQ21SData; heatmaps work without MeasurementIntegrationPack or Excel</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B10" s="13" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Windows Setup v1.3.5</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>AtomikSimulationEngine-Setup-v1.3.5.exe — EXE + fonts only (no Excel)</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B11" s="14" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Installer drops Excel folders</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>setup.iss no longer ships Factory Readings / shyamGuildMeasurements xlsx</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-26</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E31"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -714,7 +1213,7 @@
     <row r="2" ht="18" customHeight="1">
       <c r="A2" s="3" t="inlineStr">
         <is>
-          <t>Development window 2026-08-12 -&gt; 2026-08-21</t>
+          <t>Development window 2026-08-12 -&gt; 2026-08-21 (portable ZIP same day)</t>
         </is>
       </c>
       <c r="B2" s="2" t="n"/>
@@ -762,7 +1261,7 @@
           <t>Engine</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -789,7 +1288,7 @@
           <t>Array presets</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -816,7 +1315,7 @@
           <t>Docs / pack</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -843,7 +1342,7 @@
           <t>Archive</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -855,7 +1354,7 @@
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>version-archive/: list releases from v1.3.0; download source zip / macOS DMG / Windows EXE (standalone, not in-app)</t>
+          <t>version-archive/: releases from v1.3.0; source zip / macOS DMG / Windows ZIP (EXE+Data); local artifacts serve without Mongo</t>
         </is>
       </c>
       <c r="E8" s="8" t="inlineStr">
@@ -867,27 +1366,27 @@
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Plot tools</t>
-        </is>
-      </c>
-      <c r="B9" s="9" t="inlineStr">
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Heatmap drawing tools</t>
+          <t>Windows portable ZIP</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Select, Pan, Pencil, Eraser, Ruler, Line + colour swatch; annotations in world metres</t>
+          <t>EXE + MeasurementIntegrationPack\Data (Q21S CSVs); required for other PCs — bare EXE alone cannot load heatmaps</t>
         </is>
       </c>
       <c r="E9" s="6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -897,19 +1396,19 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
       </c>
       <c r="C10" s="8" t="inlineStr">
         <is>
-          <t>BEM / directivity field math</t>
+          <t>Heatmap drawing tools</t>
         </is>
       </c>
       <c r="D10" s="8" t="inlineStr">
         <is>
-          <t>Tightened BEM and measured-directivity field formation (commit 633fc36)</t>
+          <t>Select, Pan, Pencil, Eraser, Ruler, Line + colour swatch; annotations in world metres</t>
         </is>
       </c>
       <c r="E10" s="8" t="inlineStr">
@@ -921,49 +1420,49 @@
     <row r="11">
       <c r="A11" s="5" t="inlineStr">
         <is>
-          <t>Editing</t>
-        </is>
-      </c>
-      <c r="B11" s="9" t="inlineStr">
+          <t>Plot tools</t>
+        </is>
+      </c>
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
       </c>
       <c r="C11" s="6" t="inlineStr">
         <is>
-          <t>Undo / redo</t>
+          <t>Shapes + fill opacity</t>
         </is>
       </c>
       <c r="D11" s="6" t="inlineStr">
         <is>
-          <t>Ctrl+Z, Ctrl+Y, Ctrl+Shift+Z; letter is lowercased so Caps Lock still works; drawings, cabinets, layouts, control-panel edits</t>
+          <t>Rectangle, Square, Circle tools with opacity slider; undo/redo covers shapes</t>
         </is>
       </c>
       <c r="E11" s="6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="12">
       <c r="A12" s="7" t="inlineStr">
         <is>
-          <t>Packaging</t>
-        </is>
-      </c>
-      <c r="B12" s="10" t="inlineStr">
+          <t>Plot tools</t>
+        </is>
+      </c>
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
       </c>
       <c r="C12" s="8" t="inlineStr">
         <is>
-          <t>Windows Release exe</t>
+          <t>BEM / directivity field math</t>
         </is>
       </c>
       <c r="D12" s="8" t="inlineStr">
         <is>
-          <t>Builds\Release\Atomik Simulation Engine.exe; installer/README at v1.3.0</t>
+          <t>Tightened BEM and measured-directivity field formation (commit 633fc36)</t>
         </is>
       </c>
       <c r="E12" s="8" t="inlineStr">
@@ -975,162 +1474,162 @@
     <row r="13">
       <c r="A13" s="5" t="inlineStr">
         <is>
-          <t>DSP / UI (PS batch)</t>
-        </is>
-      </c>
-      <c r="B13" s="9" t="inlineStr">
+          <t>Editing</t>
+        </is>
+      </c>
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
       </c>
       <c r="C13" s="6" t="inlineStr">
         <is>
-          <t>IEC 1/3-octave frequencies</t>
+          <t>Undo / redo</t>
         </is>
       </c>
       <c r="D13" s="6" t="inlineStr">
         <is>
-          <t>20, 25, 31, 40, 50, 63, 80, 100, 125, 160, 200, 250, 315, 400, 500 Hz</t>
+          <t>Ctrl+Z, Ctrl+Y, Ctrl+Shift+Z; letter is lowercased so Caps Lock still works; drawings, cabinets, layouts, control-panel edits</t>
         </is>
       </c>
       <c r="E13" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>Cabinet</t>
-        </is>
-      </c>
-      <c r="B14" s="11" t="inlineStr">
-        <is>
-          <t>Changed</t>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B14" s="13" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="C14" s="8" t="inlineStr">
         <is>
-          <t>Q21S footprint 750×784×917 mm</t>
+          <t>Windows Release exe</t>
         </is>
       </c>
       <c r="D14" s="8" t="inlineStr">
         <is>
-          <t>Plan drawing + hit-test use true W×D; 1/r singularity floor = depth/2</t>
+          <t>Builds\Release\Atomik Simulation Engine.exe; installer/README at v1.3.0</t>
         </is>
       </c>
       <c r="E14" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
-          <t>Engine</t>
-        </is>
-      </c>
-      <c r="B15" s="12" t="inlineStr">
-        <is>
-          <t>Changed</t>
+          <t>DSP / UI (PS batch)</t>
+        </is>
+      </c>
+      <c r="B15" s="11" t="inlineStr">
+        <is>
+          <t>Added</t>
         </is>
       </c>
       <c r="C15" s="6" t="inlineStr">
         <is>
-          <t>Heatmap uses 2 m BEM arc</t>
+          <t>IEC 1/3-octave frequencies</t>
         </is>
       </c>
       <c r="D15" s="6" t="inlineStr">
         <is>
-          <t>Array/SPL prediction keeps far-field arc; Measured Polar can still show nearer distances</t>
+          <t>20, 25, 31, 40, 50, 63, 80, 100, 125, 160, 200, 250, 315, 400, 500 Hz</t>
         </is>
       </c>
       <c r="E15" s="6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" s="7" t="inlineStr">
         <is>
-          <t>Branding</t>
-        </is>
-      </c>
-      <c r="B16" s="11" t="inlineStr">
+          <t>Cabinet</t>
+        </is>
+      </c>
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
       </c>
       <c r="C16" s="8" t="inlineStr">
         <is>
-          <t>Product name</t>
+          <t>Q21S footprint 750×784×917 mm</t>
         </is>
       </c>
       <c r="D16" s="8" t="inlineStr">
         <is>
-          <t>Atomik Acoustic Simulation Engine -&gt; Atomik Simulation Engine; UI/PDF/CSV/installer/file version = v1.3.0</t>
+          <t>Plan drawing + hit-test use true W×D; 1/r singularity floor = depth/2</t>
         </is>
       </c>
       <c r="E16" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" s="5" t="inlineStr">
         <is>
-          <t>Branding</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B17" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
       </c>
       <c r="C17" s="6" t="inlineStr">
         <is>
-          <t>ATOMIK-only wordmark</t>
+          <t>Heatmap uses 2 m BEM arc</t>
         </is>
       </c>
       <c r="D17" s="6" t="inlineStr">
         <is>
-          <t>AUDIO line removed; Atomik_Logo_Dark.png / Atomik_Logo_Light.png</t>
+          <t>Array/SPL prediction keeps far-field arc; Measured Polar can still show nearer distances</t>
         </is>
       </c>
       <c r="E17" s="6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" s="7" t="inlineStr">
         <is>
-          <t>Header</t>
-        </is>
-      </c>
-      <c r="B18" s="11" t="inlineStr">
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
       </c>
       <c r="C18" s="8" t="inlineStr">
         <is>
-          <t>Statistics button</t>
+          <t>World 100×100 m</t>
         </is>
       </c>
       <c r="D18" s="8" t="inlineStr">
         <is>
-          <t>Stats pill renamed Statistics; width sized to the full label</t>
+          <t>Was 30×30 m in v1.0; full-grid Q21S coverage prediction</t>
         </is>
       </c>
       <c r="E18" s="8" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
@@ -1140,178 +1639,313 @@
           <t>Measurement</t>
         </is>
       </c>
-      <c r="B19" s="12" t="inlineStr">
+      <c r="B19" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
       </c>
       <c r="C19" s="6" t="inlineStr">
         <is>
-          <t>Ground Plane only</t>
+          <t>Q21S product set / native BEM Hz</t>
         </is>
       </c>
       <c r="D19" s="6" t="inlineStr">
         <is>
-          <t>Measurement UI is Ground Plane (no Room set in live UI)</t>
+          <t>Catalogue 20,29,52,81,98,153,198,256,309,352,400,401 Hz; UI Ground Plane only</t>
         </is>
       </c>
       <c r="E19" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-21</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" s="7" t="inlineStr">
         <is>
-          <t>DSP</t>
-        </is>
-      </c>
-      <c r="B20" s="11" t="inlineStr">
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
       </c>
       <c r="C20" s="8" t="inlineStr">
         <is>
-          <t>Legend / dB floor -6 dB steps</t>
+          <t>Product name</t>
         </is>
       </c>
       <c r="D20" s="8" t="inlineStr">
         <is>
-          <t>Colourbar ticks and floor slider on -6 dB; dBfloor is display range only</t>
+          <t>Atomik Acoustic Simulation Engine -&gt; Atomik Simulation Engine; UI/PDF/CSV/installer/file version = v1.3.0</t>
         </is>
       </c>
       <c r="E20" s="8" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" s="5" t="inlineStr">
         <is>
-          <t>UI</t>
-        </is>
-      </c>
-      <c r="B21" s="12" t="inlineStr">
+          <t>Branding</t>
+        </is>
+      </c>
+      <c r="B21" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
       </c>
       <c r="C21" s="6" t="inlineStr">
         <is>
-          <t>XN18-n labels + Set to Default</t>
+          <t>ATOMIK-only wordmark</t>
         </is>
       </c>
       <c r="D21" s="6" t="inlineStr">
         <is>
-          <t>Cabinet labels use hyphen; Reset renamed Set to Default</t>
+          <t>AUDIO line removed; Atomik_Logo_Dark.png / Atomik_Logo_Light.png</t>
         </is>
       </c>
       <c r="E21" s="6" t="inlineStr">
         <is>
-          <t>2026-08-12</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="7" t="inlineStr">
         <is>
-          <t>Engine</t>
-        </is>
-      </c>
-      <c r="B22" s="13" t="inlineStr">
-        <is>
-          <t>Fixed</t>
+          <t>Header</t>
+        </is>
+      </c>
+      <c r="B22" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
         </is>
       </c>
       <c r="C22" s="8" t="inlineStr">
         <is>
-          <t>No ±5 m BEM stamp on live map</t>
+          <t>Statistics button</t>
         </is>
       </c>
       <c r="D22" s="8" t="inlineStr">
         <is>
-          <t>Full 100×100 m map follows polar × inverse-square instead of a near-field island</t>
+          <t>Stats pill renamed Statistics; width sized to the full label</t>
         </is>
       </c>
       <c r="E22" s="8" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-19</t>
         </is>
       </c>
     </row>
     <row r="23">
       <c r="A23" s="5" t="inlineStr">
         <is>
-          <t>Header</t>
+          <t>Measurement</t>
         </is>
       </c>
       <c r="B23" s="14" t="inlineStr">
         <is>
-          <t>Fixed</t>
+          <t>Changed</t>
         </is>
       </c>
       <c r="C23" s="6" t="inlineStr">
         <is>
-          <t>Version no longer clips</t>
+          <t>Ground Plane only</t>
         </is>
       </c>
       <c r="D23" s="6" t="inlineStr">
         <is>
-          <t>Was showing v1... instead of v1.3.0; layout uses real logo width</t>
+          <t>Measurement UI is Ground Plane (no Room set in live UI)</t>
         </is>
       </c>
       <c r="E23" s="6" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-08-12</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="7" t="inlineStr">
         <is>
+          <t>DSP</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C24" s="8" t="inlineStr">
+        <is>
+          <t>Legend / dB floor -6 dB steps</t>
+        </is>
+      </c>
+      <c r="D24" s="8" t="inlineStr">
+        <is>
+          <t>Colourbar ticks and floor slider on -6 dB; dBfloor is display range only</t>
+        </is>
+      </c>
+      <c r="E24" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="5" t="inlineStr">
+        <is>
           <t>UI</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B25" s="14" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C25" s="6" t="inlineStr">
+        <is>
+          <t>XN18-n labels + Set to Default</t>
+        </is>
+      </c>
+      <c r="D25" s="6" t="inlineStr">
+        <is>
+          <t>Cabinet labels use hyphen; Reset renamed Set to Default</t>
+        </is>
+      </c>
+      <c r="E25" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-12</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="7" t="inlineStr">
+        <is>
+          <t>Engine</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
       </c>
-      <c r="C24" s="8" t="inlineStr">
+      <c r="C26" s="8" t="inlineStr">
+        <is>
+          <t>No ±5 m BEM stamp on live map</t>
+        </is>
+      </c>
+      <c r="D26" s="8" t="inlineStr">
+        <is>
+          <t>Full 100×100 m map follows polar × inverse-square instead of a near-field island</t>
+        </is>
+      </c>
+      <c r="E26" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="5" t="inlineStr">
+        <is>
+          <t>Windows</t>
+        </is>
+      </c>
+      <c r="B27" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C27" s="6" t="inlineStr">
+        <is>
+          <t>Q21S pack path (vs legacy D:\shayam gui)</t>
+        </is>
+      </c>
+      <c r="D27" s="6" t="inlineStr">
+        <is>
+          <t>Prefer exe/repo MeasurementIntegrationPack with Q21S_52Hz_2p0m.csv marker; avoid Factory/ShyamGuild-only legacy pack</t>
+        </is>
+      </c>
+      <c r="E27" s="6" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="7" t="inlineStr">
+        <is>
+          <t>Header</t>
+        </is>
+      </c>
+      <c r="B28" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C28" s="8" t="inlineStr">
+        <is>
+          <t>Version no longer clips</t>
+        </is>
+      </c>
+      <c r="D28" s="8" t="inlineStr">
+        <is>
+          <t>Was showing v1... instead of v1.3.0; layout uses real logo width</t>
+        </is>
+      </c>
+      <c r="E28" s="8" t="inlineStr">
+        <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="5" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B29" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C29" s="6" t="inlineStr">
         <is>
           <t>Small-screen logo</t>
         </is>
       </c>
-      <c r="D24" s="8" t="inlineStr">
+      <c r="D29" s="6" t="inlineStr">
         <is>
           <t>Header/dashboard wordmark -20%; Scale minFactor 0.78</t>
         </is>
       </c>
-      <c r="E24" s="8" t="inlineStr">
+      <c r="E29" s="6" t="inlineStr">
         <is>
           <t>2026-08-12</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="A25" s="2" t="n"/>
-      <c r="B25" s="2" t="n"/>
-      <c r="C25" s="2" t="n"/>
-      <c r="D25" s="2" t="n"/>
-      <c r="E25" s="2" t="n"/>
-    </row>
-    <row r="26">
-      <c r="A26" s="2" t="n"/>
-      <c r="B26" s="2" t="n"/>
-      <c r="C26" s="2" t="n"/>
-      <c r="D26" s="2" t="n"/>
-      <c r="E26" s="2" t="n"/>
+    <row r="30">
+      <c r="A30" s="2" t="n"/>
+      <c r="B30" s="2" t="n"/>
+      <c r="C30" s="2" t="n"/>
+      <c r="D30" s="2" t="n"/>
+      <c r="E30" s="2" t="n"/>
+    </row>
+    <row r="31">
+      <c r="A31" s="2" t="n"/>
+      <c r="B31" s="2" t="n"/>
+      <c r="C31" s="2" t="n"/>
+      <c r="D31" s="2" t="n"/>
+      <c r="E31" s="2" t="n"/>
     </row>
   </sheetData>
-  <autoFilter ref="A4:E24"/>
+  <autoFilter ref="A4:E29"/>
   <mergeCells count="2">
     <mergeCell ref="A2:E2"/>
     <mergeCell ref="A1:E1"/>
@@ -1320,7 +1954,209 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E9"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="16" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="34" customWidth="1" min="3" max="3"/>
+    <col width="78" customWidth="1" min="4" max="4"/>
+    <col width="13" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>v1.2.x  -  Beta UI redesign (through betav1.2.3)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>~2026-07  |  Graph colors.pdf chrome between v1.1.0 and v1.3.0</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Section</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Details</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>Date</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B5" s="14" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Graph colors.pdf tokens</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Charcoal / white / ash / signal red + heatmap cool/hot stops in BrandTheme.h</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>~2026-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Brand</t>
+        </is>
+      </c>
+      <c r="B6" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Signal Red accents</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Interactive accent #ED2227 for controls (later refined in 1.3.0 ATOMIK branding)</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>~2026-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Heatmap</t>
+        </is>
+      </c>
+      <c r="B7" s="14" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Colour map + Rel. SPL chrome</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Cool/hot stops and legend chrome aligned to brand mockups</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>~2026-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B8" s="12" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Light / dark chrome</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar density, speaker markers, plot chrome, header actions</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>~2026-07</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>betav1.2.3-style Release</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Signed Windows packaging of the redesign build (see Tools/make_ui_changelog_doc.py)</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>~2026-07</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <autoFilter ref="A4:E9"/>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1398,7 +2234,7 @@
           <t>Theming &amp; Preferences</t>
         </is>
       </c>
-      <c r="B5" s="9" t="inlineStr">
+      <c r="B5" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1425,7 +2261,7 @@
           <t>Theming &amp; Preferences</t>
         </is>
       </c>
-      <c r="B6" s="10" t="inlineStr">
+      <c r="B6" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1452,7 +2288,7 @@
           <t>Theming &amp; Preferences</t>
         </is>
       </c>
-      <c r="B7" s="9" t="inlineStr">
+      <c r="B7" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1479,7 +2315,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B8" s="10" t="inlineStr">
+      <c r="B8" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1506,7 +2342,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B9" s="9" t="inlineStr">
+      <c r="B9" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1533,7 +2369,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B10" s="10" t="inlineStr">
+      <c r="B10" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1560,7 +2396,7 @@
           <t>Heatmap Export</t>
         </is>
       </c>
-      <c r="B11" s="9" t="inlineStr">
+      <c r="B11" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1587,7 +2423,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B12" s="10" t="inlineStr">
+      <c r="B12" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1614,7 +2450,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B13" s="9" t="inlineStr">
+      <c r="B13" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1641,7 +2477,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B14" s="10" t="inlineStr">
+      <c r="B14" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1668,7 +2504,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B15" s="9" t="inlineStr">
+      <c r="B15" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1695,7 +2531,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B16" s="10" t="inlineStr">
+      <c r="B16" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1722,7 +2558,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B17" s="9" t="inlineStr">
+      <c r="B17" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1749,7 +2585,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B18" s="10" t="inlineStr">
+      <c r="B18" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1776,7 +2612,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B19" s="9" t="inlineStr">
+      <c r="B19" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1803,7 +2639,7 @@
           <t>Array Presets</t>
         </is>
       </c>
-      <c r="B20" s="10" t="inlineStr">
+      <c r="B20" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1830,7 +2666,7 @@
           <t>Array Presets</t>
         </is>
       </c>
-      <c r="B21" s="9" t="inlineStr">
+      <c r="B21" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1857,7 +2693,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B22" s="10" t="inlineStr">
+      <c r="B22" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1884,7 +2720,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B23" s="9" t="inlineStr">
+      <c r="B23" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1911,7 +2747,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B24" s="10" t="inlineStr">
+      <c r="B24" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1938,7 +2774,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B25" s="9" t="inlineStr">
+      <c r="B25" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1965,7 +2801,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B26" s="10" t="inlineStr">
+      <c r="B26" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1992,7 +2828,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B27" s="9" t="inlineStr">
+      <c r="B27" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2019,7 +2855,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B28" s="10" t="inlineStr">
+      <c r="B28" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2046,7 +2882,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B29" s="9" t="inlineStr">
+      <c r="B29" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2073,7 +2909,7 @@
           <t>Branding &amp; Installer</t>
         </is>
       </c>
-      <c r="B30" s="10" t="inlineStr">
+      <c r="B30" s="13" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2100,7 +2936,7 @@
           <t>Branding &amp; Installer</t>
         </is>
       </c>
-      <c r="B31" s="9" t="inlineStr">
+      <c r="B31" s="11" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2127,7 +2963,7 @@
           <t>Versioning</t>
         </is>
       </c>
-      <c r="B32" s="11" t="inlineStr">
+      <c r="B32" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2154,7 +2990,7 @@
           <t>Color system</t>
         </is>
       </c>
-      <c r="B33" s="12" t="inlineStr">
+      <c r="B33" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2181,7 +3017,7 @@
           <t>Measured directivity</t>
         </is>
       </c>
-      <c r="B34" s="11" t="inlineStr">
+      <c r="B34" s="12" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2208,7 +3044,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B35" s="12" t="inlineStr">
+      <c r="B35" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2235,7 +3071,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B36" s="13" t="inlineStr">
+      <c r="B36" s="10" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2262,7 +3098,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B37" s="14" t="inlineStr">
+      <c r="B37" s="9" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2289,7 +3125,7 @@
           <t>Recent Projects</t>
         </is>
       </c>
-      <c r="B38" s="13" t="inlineStr">
+      <c r="B38" s="10" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2316,7 +3152,7 @@
           <t>Installer</t>
         </is>
       </c>
-      <c r="B39" s="14" t="inlineStr">
+      <c r="B39" s="9" t="inlineStr">
         <is>
           <t>Fixed</t>
         </is>
@@ -2361,7 +3197,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2555,13 +3391,13 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:B17"/>
+  <dimension ref="A1:B19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -2711,34 +3547,58 @@
     <row r="14">
       <c r="A14" s="7" t="inlineStr">
         <is>
-          <t>2026-08-19</t>
+          <t>2026-07 (approx)</t>
         </is>
       </c>
       <c r="B14" s="8" t="inlineStr">
         <is>
-          <t>v1.3.0 Windows build: Atomik Simulation Engine rename, ATOMIK-only logo, header v1.3.0 fix, Ctrl+Z/Y, Statistics button, single Release exe</t>
+          <t>v1.2.x beta UI redesign (Graph colors.pdf → betav1.2.3 packaging)</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" s="5" t="inlineStr">
         <is>
+          <t>2026-08-19</t>
+        </is>
+      </c>
+      <c r="B15" s="6" t="inlineStr">
+        <is>
+          <t>v1.3.0 Windows build: Atomik Simulation Engine rename, ATOMIK-only logo, header v1.3.0 fix, Ctrl+Z/Y, Statistics button, single Release exe</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" s="7" t="inlineStr">
+        <is>
           <t>2026-08-21</t>
         </is>
       </c>
-      <c r="B15" s="6" t="inlineStr">
-        <is>
-          <t>Q21S BEM polar×1/r, cardioid preset, cabinet size, heatmap docs/zip, version archive; CHANGELOG date → 2026-08-21</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" s="2" t="n"/>
-      <c r="B16" s="2" t="n"/>
+      <c r="B16" s="8" t="inlineStr">
+        <is>
+          <t>Q21S BEM polar×1/r, cardioid, cabinet size, heatmap docs, version archive; plot shapes + opacity</t>
+        </is>
+      </c>
     </row>
     <row r="17">
-      <c r="A17" s="2" t="n"/>
-      <c r="B17" s="2" t="n"/>
+      <c r="A17" s="5" t="inlineStr">
+        <is>
+          <t>2026-08-21</t>
+        </is>
+      </c>
+      <c r="B17" s="6" t="inlineStr">
+        <is>
+          <t>Windows Q21S data-path fix + portable ZIP (EXE+MeasurementIntegrationPack); archive Windows = ZIP</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" s="2" t="n"/>
+      <c r="B18" s="2" t="n"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="n"/>
+      <c r="B19" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Release v1.3.7: gain fix, text box, clean slate, and drawing UX.
Co-authored-by: Cursor <cursoragent@cursor.com>
</commit_message>
<xml_diff>
--- a/ShyamGui/CHANGELOG.xlsx
+++ b/ShyamGui/CHANGELOG.xlsx
@@ -8,18 +8,19 @@
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Overview" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.6 Changes" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.5 Changes" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.0 Changes" sheetId="4" state="visible" r:id="rId4"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.2.x Beta UI" sheetId="5" state="visible" r:id="rId5"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.1.0 Changes" sheetId="6" state="visible" r:id="rId6"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.0.0 Baseline" sheetId="7" state="visible" r:id="rId7"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.7 Changes" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.6 Changes" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.5 Changes" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.3.0 Changes" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.2.x Beta UI" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.1.0 Changes" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="v1.0.0 Baseline" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Timeline" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'v1.3.0 Changes'!$A$4:$E$29</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'v1.2.x Beta UI'!$A$4:$E$9</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'v1.1.0 Changes'!$A$4:$E$39</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="4" hidden="1">'v1.3.0 Changes'!$A$4:$E$29</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'v1.2.x Beta UI'!$A$4:$E$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'v1.1.0 Changes'!$A$4:$E$39</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -170,13 +171,13 @@
     <xf numFmtId="0" fontId="7" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="left" vertical="top" wrapText="1"/>
-    </xf>
     <xf numFmtId="0" fontId="7" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="8" fillId="5" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="top" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -544,7 +545,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D12"/>
+  <dimension ref="A1:D13"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -604,146 +605,168 @@
     <row r="5">
       <c r="A5" s="5" t="inlineStr">
         <is>
-          <t>1.3.6</t>
+          <t>1.3.7</t>
         </is>
       </c>
       <c r="B5" s="6" t="inlineStr">
         <is>
-          <t>2026-08-31</t>
+          <t>2026-09-02</t>
         </is>
       </c>
       <c r="C5" s="6" t="inlineStr">
         <is>
-          <t>Mic snap + shape-edge tak</t>
+          <t>Gain fix + text box + drawing UX</t>
         </is>
       </c>
       <c r="D5" s="6" t="inlineStr">
         <is>
-          <t>Restored original mic Drag::Mic ring snap; tak when drawings meet edge-to-edge; start.md for build/run; v1.3.6 Windows Release</t>
+          <t>Gain slider affects SPL again; sidebar Delete removes all selected speakers; text box annotations (fill + rotate); clean slate on first open; Range off by default; Esc/Line/Shape-menu fixes; command terminal; delay max 10 ms; v1.3.7 Windows Release</t>
         </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>1.3.5</t>
+          <t>1.3.6</t>
         </is>
       </c>
       <c r="B6" s="8" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-31</t>
         </is>
       </c>
       <c r="C6" s="8" t="inlineStr">
         <is>
-          <t>Mic tool + embedded Q21S Setup</t>
+          <t>Mic snap + shape-edge tak</t>
         </is>
       </c>
       <c r="D6" s="8" t="inlineStr">
         <is>
-          <t>Virtual mics, FR floating window, Show Degrees, tak snap sound; Q21S CSVs baked into EXE; Windows Setup without Excel/Data folder</t>
+          <t>Restored original mic Drag::Mic ring snap; tak when drawings meet edge-to-edge; start.md for build/run; v1.3.6 Windows Release</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>1.3.0</t>
+          <t>1.3.5</t>
         </is>
       </c>
       <c r="B7" s="6" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-08-26</t>
         </is>
       </c>
       <c r="C7" s="6" t="inlineStr">
         <is>
-          <t>Q21S BEM heatmap + Windows/mac product</t>
+          <t>Mic tool + embedded Q21S Setup</t>
         </is>
       </c>
       <c r="D7" s="6" t="inlineStr">
         <is>
-          <t>BEM polar×1/r full-grid SPL, cardioid, Q21S 750×784×917 mm, plot tools/shapes, undo/redo, ATOMIK branding, version archive, Windows portable ZIP (EXE+Data)</t>
+          <t>Virtual mics, FR floating window, Show Degrees, tak snap sound; Q21S CSVs baked into EXE; Windows Setup without Excel/Data folder</t>
         </is>
       </c>
     </row>
     <row r="8">
       <c r="A8" s="7" t="inlineStr">
         <is>
-          <t>1.2.x</t>
+          <t>1.3.0</t>
         </is>
       </c>
       <c r="B8" s="8" t="inlineStr">
         <is>
-          <t>~2026-07</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="C8" s="8" t="inlineStr">
         <is>
-          <t>Beta UI redesign (betav1.2.3)</t>
+          <t>Q21S BEM heatmap + Windows/mac product</t>
         </is>
       </c>
       <c r="D8" s="8" t="inlineStr">
         <is>
-          <t>Graph colors.pdf chrome: brand tokens, heatmap colour stops, light/dark sidebar; packaged as betav1.2.3-style Release</t>
+          <t>BEM polar×1/r full-grid SPL, cardioid, Q21S 750×784×917 mm, plot tools/shapes, undo/redo, ATOMIK branding, version archive, Windows portable ZIP (EXE+Data)</t>
         </is>
       </c>
     </row>
     <row r="9">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>1.1.0</t>
+          <t>1.2.x</t>
         </is>
       </c>
       <c r="B9" s="6" t="inlineStr">
         <is>
-          <t>2026-06-29</t>
+          <t>~2026-07</t>
         </is>
       </c>
       <c r="C9" s="6" t="inlineStr">
         <is>
-          <t>Major feature + UX release</t>
+          <t>Beta UI redesign (betav1.2.3)</t>
         </is>
       </c>
       <c r="D9" s="6" t="inlineStr">
         <is>
-          <t>Theming, project dashboard/.atmk, heatmap + PDF export, grid/CAD-DXF, array presets, dual datasets, responsive window, branded installer</t>
+          <t>Graph colors.pdf chrome: brand tokens, heatmap colour stops, light/dark sidebar; packaged as betav1.2.3-style Release</t>
         </is>
       </c>
     </row>
     <row r="10">
       <c r="A10" s="7" t="inlineStr">
         <is>
+          <t>1.1.0</t>
+        </is>
+      </c>
+      <c r="B10" s="8" t="inlineStr">
+        <is>
+          <t>2026-06-29</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Major feature + UX release</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Theming, project dashboard/.atmk, heatmap + PDF export, grid/CAD-DXF, array presets, dual datasets, responsive window, branded installer</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
           <t>1.0.0</t>
         </is>
       </c>
-      <c r="B10" s="8" t="inlineStr">
+      <c r="B11" s="6" t="inlineStr">
         <is>
           <t>2026-06-22</t>
         </is>
       </c>
-      <c r="C10" s="8" t="inlineStr">
+      <c r="C11" s="6" t="inlineStr">
         <is>
           <t>Initial baseline</t>
         </is>
       </c>
-      <c r="D10" s="8" t="inlineStr">
+      <c r="D11" s="6" t="inlineStr">
         <is>
           <t>Dual-subwoofer (XN18) prediction &amp; visualisation in a 30x30 m world; measured directivity added 2026-06-24</t>
         </is>
       </c>
-    </row>
-    <row r="11">
-      <c r="A11" s="2" t="n"/>
-      <c r="B11" s="2" t="n"/>
-      <c r="C11" s="2" t="n"/>
-      <c r="D11" s="2" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="2" t="n"/>
       <c r="B12" s="2" t="n"/>
       <c r="C12" s="2" t="n"/>
       <c r="D12" s="2" t="n"/>
+    </row>
+    <row r="13">
+      <c r="A13" s="2" t="n"/>
+      <c r="B13" s="2" t="n"/>
+      <c r="C13" s="2" t="n"/>
+      <c r="D13" s="2" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
@@ -755,6 +778,342 @@
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="A1:E14"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="14" customWidth="1" min="1" max="1"/>
+    <col width="10" customWidth="1" min="2" max="2"/>
+    <col width="28" customWidth="1" min="3" max="3"/>
+    <col width="72" customWidth="1" min="4" max="4"/>
+    <col width="12" customWidth="1" min="5" max="5"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="34" customHeight="1">
+      <c r="A1" s="1" t="inlineStr">
+        <is>
+          <t>v1.3.7  -  Detailed Changes</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="18" customHeight="1">
+      <c r="A2" s="3" t="inlineStr">
+        <is>
+          <t>2026-09-02  |  Gain fix + text box + clean slate + drawing UX</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="22" customHeight="1">
+      <c r="A4" s="4" t="inlineStr">
+        <is>
+          <t>Area</t>
+        </is>
+      </c>
+      <c r="B4" s="4" t="inlineStr">
+        <is>
+          <t>Type</t>
+        </is>
+      </c>
+      <c r="C4" s="4" t="inlineStr">
+        <is>
+          <t>Item</t>
+        </is>
+      </c>
+      <c r="D4" s="4" t="inlineStr">
+        <is>
+          <t>Detail</t>
+        </is>
+      </c>
+      <c r="E4" s="4" t="inlineStr">
+        <is>
+          <t>When</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="A5" s="5" t="inlineStr">
+        <is>
+          <t>Speakers</t>
+        </is>
+      </c>
+      <c r="B5" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C5" s="6" t="inlineStr">
+        <is>
+          <t>Gain (dB) affects SPL</t>
+        </is>
+      </c>
+      <c r="D5" s="6" t="inlineStr">
+        <is>
+          <t>Unity-gain reference normalisation; per-speaker level and array balance visible on heatmap</t>
+        </is>
+      </c>
+      <c r="E5" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="7" t="inlineStr">
+        <is>
+          <t>Speakers</t>
+        </is>
+      </c>
+      <c r="B6" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C6" s="8" t="inlineStr">
+        <is>
+          <t>Delete all selected</t>
+        </is>
+      </c>
+      <c r="D6" s="8" t="inlineStr">
+        <is>
+          <t>Sidebar Delete removes every speaker in plot multi-selection, not just primary unit</t>
+        </is>
+      </c>
+      <c r="E6" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="5" t="inlineStr">
+        <is>
+          <t>Plot tools</t>
+        </is>
+      </c>
+      <c r="B7" s="9" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C7" s="6" t="inlineStr">
+        <is>
+          <t>Line first stroke</t>
+        </is>
+      </c>
+      <c r="D7" s="6" t="inlineStr">
+        <is>
+          <t>Minimum drag distance prevents accidental micro-line consuming first click</t>
+        </is>
+      </c>
+      <c r="E7" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>Plot tools</t>
+        </is>
+      </c>
+      <c r="B8" s="10" t="inlineStr">
+        <is>
+          <t>Fixed</t>
+        </is>
+      </c>
+      <c r="C8" s="8" t="inlineStr">
+        <is>
+          <t>Esc + Shape menu</t>
+        </is>
+      </c>
+      <c r="D8" s="8" t="inlineStr">
+        <is>
+          <t>Esc returns to Select from drawing tools; cursor tool no longer opens Shape menu</t>
+        </is>
+      </c>
+      <c r="E8" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="A9" s="5" t="inlineStr">
+        <is>
+          <t>UI</t>
+        </is>
+      </c>
+      <c r="B9" s="11" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C9" s="6" t="inlineStr">
+        <is>
+          <t>Command terminal</t>
+        </is>
+      </c>
+      <c r="D9" s="6" t="inlineStr">
+        <is>
+          <t>Bottom-panel terminal replaces Phase/Arrival/STI placeholders; cls/clear supported</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="7" t="inlineStr">
+        <is>
+          <t>Plot tools</t>
+        </is>
+      </c>
+      <c r="B10" s="12" t="inlineStr">
+        <is>
+          <t>Added</t>
+        </is>
+      </c>
+      <c r="C10" s="8" t="inlineStr">
+        <is>
+          <t>Text box annotations</t>
+        </is>
+      </c>
+      <c r="D10" s="8" t="inlineStr">
+        <is>
+          <t>Shape menu Text Box; fill colour like shapes; rotation handle; double-click edit</t>
+        </is>
+      </c>
+      <c r="E10" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>Speakers</t>
+        </is>
+      </c>
+      <c r="B11" s="13" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C11" s="6" t="inlineStr">
+        <is>
+          <t>Delay slider max 10 ms</t>
+        </is>
+      </c>
+      <c r="D11" s="6" t="inlineStr">
+        <is>
+          <t>Was 50 ms; presets unchanged</t>
+        </is>
+      </c>
+      <c r="E11" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="12">
+      <c r="A12" s="7" t="inlineStr">
+        <is>
+          <t>Project</t>
+        </is>
+      </c>
+      <c r="B12" s="14" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C12" s="8" t="inlineStr">
+        <is>
+          <t>Clean slate on first open</t>
+        </is>
+      </c>
+      <c r="D12" s="8" t="inlineStr">
+        <is>
+          <t>No default speakers until user adds a Q21S unit</t>
+        </is>
+      </c>
+      <c r="E12" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
+          <t>Plot</t>
+        </is>
+      </c>
+      <c r="B13" s="13" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C13" s="6" t="inlineStr">
+        <is>
+          <t>Range off by default</t>
+        </is>
+      </c>
+      <c r="D13" s="6" t="inlineStr">
+        <is>
+          <t>Distance rings hidden until Range toggle is on</t>
+        </is>
+      </c>
+      <c r="E13" s="6" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" s="7" t="inlineStr">
+        <is>
+          <t>Packaging</t>
+        </is>
+      </c>
+      <c r="B14" s="14" t="inlineStr">
+        <is>
+          <t>Changed</t>
+        </is>
+      </c>
+      <c r="C14" s="8" t="inlineStr">
+        <is>
+          <t>Version → v1.3.7 (refresh)</t>
+        </is>
+      </c>
+      <c r="D14" s="8" t="inlineStr">
+        <is>
+          <t>App, resource, installer defines, archive HTML/json, Windows Release EXE</t>
+        </is>
+      </c>
+      <c r="E14" s="8" t="inlineStr">
+        <is>
+          <t>2026-09-02</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A2:E2"/>
+    <mergeCell ref="A1:E1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -898,7 +1257,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -928,7 +1287,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1018,7 +1377,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1072,7 +1431,7 @@
           <t>Mic tool</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1126,7 +1485,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1153,7 +1512,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B11" s="14" t="inlineStr">
+      <c r="B11" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1183,7 +1542,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet4.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -1288,7 +1647,7 @@
           <t>Array presets</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1342,7 +1701,7 @@
           <t>Archive</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1396,7 +1755,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1450,7 +1809,7 @@
           <t>Plot tools</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1504,7 +1863,7 @@
           <t>Packaging</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -1558,7 +1917,7 @@
           <t>Cabinet</t>
         </is>
       </c>
-      <c r="B16" s="12" t="inlineStr">
+      <c r="B16" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1585,7 +1944,7 @@
           <t>Engine</t>
         </is>
       </c>
-      <c r="B17" s="14" t="inlineStr">
+      <c r="B17" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1612,7 +1971,7 @@
           <t>Engine</t>
         </is>
       </c>
-      <c r="B18" s="12" t="inlineStr">
+      <c r="B18" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1639,7 +1998,7 @@
           <t>Measurement</t>
         </is>
       </c>
-      <c r="B19" s="14" t="inlineStr">
+      <c r="B19" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1666,7 +2025,7 @@
           <t>Branding</t>
         </is>
       </c>
-      <c r="B20" s="12" t="inlineStr">
+      <c r="B20" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1693,7 +2052,7 @@
           <t>Branding</t>
         </is>
       </c>
-      <c r="B21" s="14" t="inlineStr">
+      <c r="B21" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1720,7 +2079,7 @@
           <t>Header</t>
         </is>
       </c>
-      <c r="B22" s="12" t="inlineStr">
+      <c r="B22" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1747,7 +2106,7 @@
           <t>Measurement</t>
         </is>
       </c>
-      <c r="B23" s="14" t="inlineStr">
+      <c r="B23" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1774,7 +2133,7 @@
           <t>DSP</t>
         </is>
       </c>
-      <c r="B24" s="12" t="inlineStr">
+      <c r="B24" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1801,7 +2160,7 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="B25" s="14" t="inlineStr">
+      <c r="B25" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -1954,7 +2313,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet5.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2017,7 +2376,7 @@
           <t>Brand</t>
         </is>
       </c>
-      <c r="B5" s="14" t="inlineStr">
+      <c r="B5" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2044,7 +2403,7 @@
           <t>Brand</t>
         </is>
       </c>
-      <c r="B6" s="12" t="inlineStr">
+      <c r="B6" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2071,7 +2430,7 @@
           <t>Heatmap</t>
         </is>
       </c>
-      <c r="B7" s="14" t="inlineStr">
+      <c r="B7" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2098,7 +2457,7 @@
           <t>UI</t>
         </is>
       </c>
-      <c r="B8" s="12" t="inlineStr">
+      <c r="B8" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2156,7 +2515,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -2261,7 +2620,7 @@
           <t>Theming &amp; Preferences</t>
         </is>
       </c>
-      <c r="B6" s="13" t="inlineStr">
+      <c r="B6" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2315,7 +2674,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B8" s="13" t="inlineStr">
+      <c r="B8" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2369,7 +2728,7 @@
           <t>Project Workflow</t>
         </is>
       </c>
-      <c r="B10" s="13" t="inlineStr">
+      <c r="B10" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2423,7 +2782,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B12" s="13" t="inlineStr">
+      <c r="B12" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2477,7 +2836,7 @@
           <t>PDF Report</t>
         </is>
       </c>
-      <c r="B14" s="13" t="inlineStr">
+      <c r="B14" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2531,7 +2890,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B16" s="13" t="inlineStr">
+      <c r="B16" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2585,7 +2944,7 @@
           <t>Workspace / Grid / Layout</t>
         </is>
       </c>
-      <c r="B18" s="13" t="inlineStr">
+      <c r="B18" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2639,7 +2998,7 @@
           <t>Array Presets</t>
         </is>
       </c>
-      <c r="B20" s="13" t="inlineStr">
+      <c r="B20" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2693,7 +3052,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B22" s="13" t="inlineStr">
+      <c r="B22" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2747,7 +3106,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B24" s="13" t="inlineStr">
+      <c r="B24" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2801,7 +3160,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B26" s="13" t="inlineStr">
+      <c r="B26" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2855,7 +3214,7 @@
           <t>Responsive UI</t>
         </is>
       </c>
-      <c r="B28" s="13" t="inlineStr">
+      <c r="B28" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2909,7 +3268,7 @@
           <t>Branding &amp; Installer</t>
         </is>
       </c>
-      <c r="B30" s="13" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>Added</t>
         </is>
@@ -2963,7 +3322,7 @@
           <t>Versioning</t>
         </is>
       </c>
-      <c r="B32" s="12" t="inlineStr">
+      <c r="B32" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -2990,7 +3349,7 @@
           <t>Color system</t>
         </is>
       </c>
-      <c r="B33" s="14" t="inlineStr">
+      <c r="B33" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -3017,7 +3376,7 @@
           <t>Measured directivity</t>
         </is>
       </c>
-      <c r="B34" s="12" t="inlineStr">
+      <c r="B34" s="14" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -3044,7 +3403,7 @@
           <t>Measurement Datasets</t>
         </is>
       </c>
-      <c r="B35" s="14" t="inlineStr">
+      <c r="B35" s="13" t="inlineStr">
         <is>
           <t>Changed</t>
         </is>
@@ -3197,7 +3556,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>
@@ -3391,7 +3750,7 @@
 </worksheet>
 </file>
 
-<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>
     <outlinePr summaryBelow="1" summaryRight="1"/>

</xml_diff>